<commit_message>
added image on home page
</commit_message>
<xml_diff>
--- a/excels/Cep.xlsx
+++ b/excels/Cep.xlsx
@@ -5,16 +5,17 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CED TD-11\Downloads\fmain\NITW-Transportation-Division-main\excels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CED TD-11\Downloads\mainnn\NITW-Transportation-Division-main\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12180" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14370" windowHeight="10350" firstSheet="3" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Seminars" sheetId="1" r:id="rId1"/>
     <sheet name="Training" sheetId="2" r:id="rId2"/>
     <sheet name="FacultyDevelopmentPrograms" sheetId="3" r:id="rId3"/>
+    <sheet name="ShortTermTrainingPrograms" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="276">
   <si>
     <t>S.No</t>
   </si>
@@ -764,6 +765,96 @@
   </si>
   <si>
     <t>Enhanced academic delivery skills</t>
+  </si>
+  <si>
+    <t>Package Title</t>
+  </si>
+  <si>
+    <t>Author</t>
+  </si>
+  <si>
+    <t>Package Type</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>Level</t>
+  </si>
+  <si>
+    <t>A Five Day Executive Development Program on Design of Flexible and Rigid Pavements for Rural Roads</t>
+  </si>
+  <si>
+    <t>Dr. S. Shankar, Dr. Venkaiah Chowdary, Prof. C.S.R.K. Prasad</t>
+  </si>
+  <si>
+    <t>Sponsored by National Rural Infrastructure Development Agency, Ministry of Rural Development, Govt. of India</t>
+  </si>
+  <si>
+    <t>Panchayat Raj and PWD Engineers</t>
+  </si>
+  <si>
+    <t>New Technology Initiatives in Rural Roads and Use of Marginal Materials</t>
+  </si>
+  <si>
+    <t>Planning, Design, Construction of Culverts and Bridges, New Technology Initiatives in Rural Roads and Use of Marginal Materials</t>
+  </si>
+  <si>
+    <t>Dr. S. Shankar, Prof. G. Rajesh Kumar, Prof. C.S.R.K. Prasad</t>
+  </si>
+  <si>
+    <t>Innovative Technologies for Rural Road Construction.</t>
+  </si>
+  <si>
+    <t>Dr. S. Shankar, Prof. C.S.R.K. Prasad, Dr. Venkaiah Chowdary</t>
+  </si>
+  <si>
+    <t>Construction and Quality Control of Flexible and Rigid Pavements</t>
+  </si>
+  <si>
+    <t>Dr. S. Shankar, Prof. CSRK Prasad, and Dr. Venkaiah Chowdary</t>
+  </si>
+  <si>
+    <t>Training for Newly Inducted Officers in PMGSY</t>
+  </si>
+  <si>
+    <t>Dr. S. Shankar Prof. C.S.R.K. Prasad Prof. Venkaiah Chowdary</t>
+  </si>
+  <si>
+    <t>Planning, Design and Construction of Minor Bridges and Culverts</t>
+  </si>
+  <si>
+    <t>Dr S. Shankar, Prof. CSRK Prasad; Prof. G Rajesh Kumar</t>
+  </si>
+  <si>
+    <t>New Technology Initiatives in Rural Roads Including Use of Marginal Materials</t>
+  </si>
+  <si>
+    <t>Preparation of DPRs for Rural Road Projects</t>
+  </si>
+  <si>
+    <t>Design of Flexible and Rigid Pavements for Rural Roads</t>
+  </si>
+  <si>
+    <t>Dr. S. Shankar Prof. CSRK Prasad Prof. Venkaiah Chowdary</t>
+  </si>
+  <si>
+    <t>Ground Improvement Techniques for Rural Roads</t>
+  </si>
+  <si>
+    <t>Dr. S. Shankar, Prof. C.S.R.K. Prasad., Prof. V. Ramana Murthy</t>
+  </si>
+  <si>
+    <t>Resilient Technologies for Rural Roads</t>
+  </si>
+  <si>
+    <t>Socio-Economic Impacts of Rural Roads</t>
+  </si>
+  <si>
+    <t>Dr. S. Shankar, Dr. B. Raguram Prof. C.S.R.K. Prasad</t>
+  </si>
+  <si>
+    <t>Rural Road Construction Methods</t>
   </si>
 </sst>
 </file>
@@ -2403,4 +2494,314 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>246</v>
+      </c>
+      <c r="C1" t="s">
+        <v>247</v>
+      </c>
+      <c r="D1" t="s">
+        <v>248</v>
+      </c>
+      <c r="E1" t="s">
+        <v>249</v>
+      </c>
+      <c r="F1" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>251</v>
+      </c>
+      <c r="C2" t="s">
+        <v>252</v>
+      </c>
+      <c r="D2" t="s">
+        <v>253</v>
+      </c>
+      <c r="E2">
+        <v>2021</v>
+      </c>
+      <c r="F2" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>255</v>
+      </c>
+      <c r="C3" t="s">
+        <v>252</v>
+      </c>
+      <c r="D3" t="s">
+        <v>253</v>
+      </c>
+      <c r="E3">
+        <v>2021</v>
+      </c>
+      <c r="F3" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>256</v>
+      </c>
+      <c r="C4" t="s">
+        <v>257</v>
+      </c>
+      <c r="D4" t="s">
+        <v>253</v>
+      </c>
+      <c r="E4">
+        <v>2022</v>
+      </c>
+      <c r="F4" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>258</v>
+      </c>
+      <c r="C5" t="s">
+        <v>259</v>
+      </c>
+      <c r="D5" t="s">
+        <v>253</v>
+      </c>
+      <c r="E5">
+        <v>2022</v>
+      </c>
+      <c r="F5" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>260</v>
+      </c>
+      <c r="C6" t="s">
+        <v>261</v>
+      </c>
+      <c r="D6" t="s">
+        <v>253</v>
+      </c>
+      <c r="E6">
+        <v>2022</v>
+      </c>
+      <c r="F6" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>262</v>
+      </c>
+      <c r="C7" t="s">
+        <v>263</v>
+      </c>
+      <c r="D7" t="s">
+        <v>253</v>
+      </c>
+      <c r="E7">
+        <v>2022</v>
+      </c>
+      <c r="F7" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>264</v>
+      </c>
+      <c r="C8" t="s">
+        <v>265</v>
+      </c>
+      <c r="D8" t="s">
+        <v>253</v>
+      </c>
+      <c r="E8">
+        <v>2022</v>
+      </c>
+      <c r="F8" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>266</v>
+      </c>
+      <c r="C9" t="s">
+        <v>263</v>
+      </c>
+      <c r="D9" t="s">
+        <v>253</v>
+      </c>
+      <c r="E9">
+        <v>2022</v>
+      </c>
+      <c r="F9" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>267</v>
+      </c>
+      <c r="C10" t="s">
+        <v>263</v>
+      </c>
+      <c r="D10" t="s">
+        <v>253</v>
+      </c>
+      <c r="E10">
+        <v>2022</v>
+      </c>
+      <c r="F10" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>268</v>
+      </c>
+      <c r="C11" t="s">
+        <v>269</v>
+      </c>
+      <c r="D11" t="s">
+        <v>253</v>
+      </c>
+      <c r="E11">
+        <v>2023</v>
+      </c>
+      <c r="F11" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>270</v>
+      </c>
+      <c r="C12" t="s">
+        <v>271</v>
+      </c>
+      <c r="D12" t="s">
+        <v>253</v>
+      </c>
+      <c r="E12">
+        <v>2025</v>
+      </c>
+      <c r="F12" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>272</v>
+      </c>
+      <c r="C13" t="s">
+        <v>252</v>
+      </c>
+      <c r="D13" t="s">
+        <v>253</v>
+      </c>
+      <c r="E13">
+        <v>2025</v>
+      </c>
+      <c r="F13" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>273</v>
+      </c>
+      <c r="C14" t="s">
+        <v>274</v>
+      </c>
+      <c r="D14" t="s">
+        <v>253</v>
+      </c>
+      <c r="E14">
+        <v>2025</v>
+      </c>
+      <c r="F14" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>275</v>
+      </c>
+      <c r="C15" t="s">
+        <v>252</v>
+      </c>
+      <c r="D15" t="s">
+        <v>253</v>
+      </c>
+      <c r="E15">
+        <v>2024</v>
+      </c>
+      <c r="F15" t="s">
+        <v>254</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
updated CEP,REsearch,faculty excel data
</commit_message>
<xml_diff>
--- a/excels/Cep.xlsx
+++ b/excels/Cep.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{114B4431-7E62-4FAB-B2D9-3049523EA2E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACD4E24C-D157-4DDD-A33D-B344723E05E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Seminars" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="44">
   <si>
     <t>S.No</t>
   </si>
@@ -63,21 +63,9 @@
     <t>Expected Outcomes</t>
   </si>
   <si>
-    <t>Package Title</t>
-  </si>
-  <si>
-    <t>Author</t>
-  </si>
-  <si>
-    <t>Package Type</t>
-  </si>
-  <si>
     <t>Year</t>
   </si>
   <si>
-    <t>Level</t>
-  </si>
-  <si>
     <t>A Five Day Executive Development Program on Design of Flexible and Rigid Pavements for Rural Roads</t>
   </si>
   <si>
@@ -154,6 +142,24 @@
   </si>
   <si>
     <t>N/A</t>
+  </si>
+  <si>
+    <t>Name of the Presenter</t>
+  </si>
+  <si>
+    <t>Title of the Program</t>
+  </si>
+  <si>
+    <t>Coordinators</t>
+  </si>
+  <si>
+    <t>Sponsored Agency</t>
+  </si>
+  <si>
+    <t>Budget</t>
+  </si>
+  <si>
+    <t>No.of Participants</t>
   </si>
 </sst>
 </file>
@@ -509,7 +515,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
@@ -520,7 +526,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -529,7 +535,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -538,7 +544,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -547,7 +553,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -556,7 +562,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -565,7 +571,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -574,7 +580,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -583,7 +589,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -592,7 +598,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -601,7 +607,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -610,7 +616,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -619,7 +625,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -628,7 +634,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -719,7 +725,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -728,7 +734,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -737,7 +743,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -746,7 +752,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -755,7 +761,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -764,7 +770,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -773,7 +779,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -782,7 +788,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -791,7 +797,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -800,7 +806,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -1098,7 +1104,7 @@
     </row>
     <row r="2" spans="1:5" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1107,7 +1113,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -1116,7 +1122,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -1125,7 +1131,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -1134,7 +1140,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -1143,7 +1149,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -1152,7 +1158,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -1161,7 +1167,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -1170,7 +1176,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -1179,7 +1185,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -1263,307 +1269,310 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1" t="s">
         <v>11</v>
       </c>
-      <c r="C1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E1" t="s">
-        <v>14</v>
-      </c>
       <c r="F1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+      <c r="G1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E2">
         <v>2021</v>
       </c>
       <c r="F2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E3">
         <v>2021</v>
       </c>
       <c r="F3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D4" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E4">
         <v>2022</v>
       </c>
       <c r="F4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C5" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D5" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E5">
         <v>2022</v>
       </c>
       <c r="F5" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C6" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D6" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E6">
         <v>2022</v>
       </c>
       <c r="F6" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C7" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D7" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E7">
         <v>2022</v>
       </c>
       <c r="F7" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C8" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="D8" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E8">
         <v>2022</v>
       </c>
       <c r="F8" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C9" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D9" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E9">
         <v>2022</v>
       </c>
       <c r="F9" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C10" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D10" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E10">
         <v>2022</v>
       </c>
       <c r="F10" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C11" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D11" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E11">
         <v>2023</v>
       </c>
       <c r="F11" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C12" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D12" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E12">
         <v>2025</v>
       </c>
       <c r="F12" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C13" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D13" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E13">
         <v>2025</v>
       </c>
       <c r="F13" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C14" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D14" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E14">
         <v>2025</v>
       </c>
       <c r="F14" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C15" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D15" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E15">
         <v>2024</v>
       </c>
       <c r="F15" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>